<commit_message>
test(campaign): finalize G04 post-closure metadata
</commit_message>
<xml_diff>
--- a/Matrice_semplificata_G04_allineata.xlsx
+++ b/Matrice_semplificata_G04_allineata.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R7a707ee53e464fa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Run_G02" sheetId="2" r:id="Rff11764b300d4f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Riepilogo_config" sheetId="3" r:id="Rd3c03a9f3b3949a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Storico" sheetId="4" r:id="R71ccdf604f54469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Legenda" sheetId="5" r:id="Re47342a244e243bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Risultati_G03" sheetId="6" r:id="R5e9ef292448b4a8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Risultati_G04" sheetId="7" r:id="R0f12f9761d794e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Dashboard" sheetId="1" r:id="R0b5e5686289f450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Run_G02" sheetId="2" r:id="R3cbd662cf5024a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Riepilogo_config" sheetId="3" r:id="Rf906d18998bb49f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Storico" sheetId="4" r:id="R11f7322f55b64f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Legenda" sheetId="5" r:id="R019adc512d5e4f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Risultati_G03" sheetId="6" r:id="R7f2812c300174e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Risultati_G04" sheetId="7" r:id="Rfbc7ddb156d64b97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1553,7 +1553,7 @@
         <x:v>Avanzamento G04</x:v>
       </x:c>
       <x:c r="B15" s="60" t="str">
-        <x:v>Chiusura documentale pronta; commit/push tramite script</x:v>
+        <x:v>Chiusura formale completata e pubblicata al commit 4ab01845f772640398c25ba7f565ec857d284052</x:v>
       </x:c>
       <x:c r="C15" s="46"/>
       <x:c r="D15" s="46" t="n">
@@ -1577,7 +1577,7 @@
         <x:v>Prossima attività</x:v>
       </x:c>
       <x:c r="B16" s="46" t="str">
-        <x:v>Eseguire lo script di chiusura e verificare l'output</x:v>
+        <x:v>Preparare e verificare il preflight G05; non avviare run prima del controllo.</x:v>
       </x:c>
       <x:c r="C16" s="46"/>
       <x:c r="D16" s="46" t="n">
@@ -4677,7 +4677,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f7a0bd637904e0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07f783cf8a8f4a70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6316,7 +6316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R528757545b134546"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56a4ed511cb34056"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>